<commit_message>
feat: snapshot W36–W37 pricing, reconciliation, and sales materials
Refresh L3a/custom quotes and OpenAI quote tooling; add TokenHub Aug and Seedance Sep recon packs (incl. external sheet); land Tencent cloud service-fee workbooks, weekly notes, and A4 flyer/sales-kit updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/Trinity模型报价表.xlsx
+++ b/pricing/output/Trinity模型报价表.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -624,42 +624,42 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>gpt-5</t>
+          <t>gpt-5.5</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>GPT-5</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>8.5折</t>
+          <t>6.2折</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>8.2折</t>
+          <t>6折</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>7.2折</t>
+          <t>5.5折</t>
         </is>
       </c>
     </row>
@@ -668,42 +668,42 @@
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>gpt-5-nano</t>
+          <t>gpt-5.6-luna</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>GPT-5 Nano</t>
+          <t>GPT-5.6 Luna</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>8.5折</t>
+          <t>6.2折</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>8.2折</t>
+          <t>6折</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>7.2折</t>
+          <t>5.5折</t>
         </is>
       </c>
     </row>
@@ -712,12 +712,12 @@
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.1</t>
+          <t>gpt-5</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.1</t>
+          <t>GPT-5</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -756,27 +756,27 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.2</t>
+          <t>gpt-5-nano</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.2</t>
+          <t>GPT-5 Nano</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -800,27 +800,27 @@
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.3-codex</t>
+          <t>gpt-5.1</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.3 Codex</t>
+          <t>GPT-5.1</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -844,27 +844,27 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.4</t>
+          <t>gpt-5.2</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.4</t>
+          <t>GPT-5.2</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>15.00</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -888,27 +888,27 @@
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.4-mini</t>
+          <t>gpt-5.3-codex</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.4 Mini</t>
+          <t>GPT-5.3 Codex</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -932,27 +932,27 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.4-nano</t>
+          <t>gpt-5.4</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.4 nano</t>
+          <t>GPT-5.4</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -976,27 +976,27 @@
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.4-pro</t>
+          <t>gpt-5.4-mini</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.4 Pro</t>
+          <t>GPT-5.4 Mini</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>180.00</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1020,27 +1020,27 @@
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.5</t>
+          <t>gpt-5.4-nano</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GPT-5.4 nano</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1064,27 +1064,27 @@
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>gpt-5.6-luna</t>
+          <t>gpt-5.4-pro</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna</t>
+          <t>GPT-5.4 Pro</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>180.00</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1949,7 +1949,7 @@
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="n"/>
+      <c r="B33" s="6" t="n"/>
       <c r="C33" s="4" t="inlineStr">
         <is>
           <t>gemini-3.5-flash-lite</t>
@@ -1993,141 +1993,137 @@
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>DeepSeek</t>
-        </is>
-      </c>
+      <c r="B34" s="7" t="n"/>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>deepseek-v3.2</t>
+          <t>gemini-3.8-flash</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>DeepSeek V3.2</t>
+          <t>Gemini 3.8 Flash</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>9.2折</t>
+          <t>9折</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>8.8折</t>
+          <t>8.7折</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>7.8折</t>
+          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
-      <c r="B35" s="7" t="n"/>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash-fast</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Flash Fast</t>
+          <t>DeepSeek V4 Flash Direct</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>9.2折</t>
+          <t>8.2折</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>8.8折</t>
+          <t>7.6折</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>7.8折</t>
+          <t>6.7折</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>月之暗面</t>
-        </is>
-      </c>
+      <c r="B36" s="6" t="n"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>deepseek-v4-pro</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Kimi K3</t>
+          <t>DeepSeek V4 Pro Direct</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>15.39</t>
+          <t>3.96</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>6.6折</t>
+          <t>8.2折</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>6.3折</t>
+          <t>7.6折</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>5.8折</t>
+          <t>6.7折</t>
         </is>
       </c>
     </row>
@@ -2136,27 +2132,27 @@
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>kimi-k2.5</t>
+          <t>deepseek-v3.2</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Kimi K2.5</t>
+          <t>DeepSeek V3.2</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -2177,30 +2173,30 @@
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
+      <c r="B38" s="7" t="n"/>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>deepseek-v4-flash-fast</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Kimi K2.6</t>
+          <t>DeepSeek V4 Flash Fast</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -2221,7 +2217,11 @@
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
-      <c r="B39" s="7" t="n"/>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>月之暗面</t>
+        </is>
+      </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
           <t>kimi-k2.7-code</t>
@@ -2265,63 +2265,63 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>MiniMax</t>
-        </is>
-      </c>
+      <c r="B40" s="7" t="n"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>minimax-m2.5</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>MiniMax M2.5</t>
+          <t>Kimi K3</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>15.39</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>9.2折</t>
+          <t>9折</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>8.8折</t>
+          <t>8.7折</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>7.8折</t>
+          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>minimax-m2.7</t>
+          <t>minimax-m2.5</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>MiniMax M2.7</t>
+          <t>MiniMax M2.5</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -2357,15 +2357,15 @@
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
-      <c r="B42" s="7" t="n"/>
+      <c r="B42" s="6" t="n"/>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>minimax-m2.7</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>MiniMax M3</t>
+          <t>MiniMax M2.7</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2401,63 +2401,63 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>智谱</t>
-        </is>
-      </c>
+      <c r="B43" s="7" t="n"/>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>glm-5.2</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>GLM-5.2</t>
+          <t>MiniMax M3</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>4.40</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>6.2折</t>
+          <t>9.2折</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>8.8折</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>5.5折</t>
+          <t>7.8折</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
-      <c r="B44" s="7" t="n"/>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>智谱</t>
+        </is>
+      </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>glm-5.3</t>
+          <t>glm-5.2</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>GLM-5.3</t>
+          <t>GLM-5.2</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2493,122 +2493,122 @@
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>阿里云·通义</t>
-        </is>
-      </c>
+      <c r="B45" s="6" t="n"/>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>qwen-flash</t>
+          <t>glm-5.3</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Qwen Flash</t>
+          <t>GLM-5.3</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>4.40</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>8.2折</t>
+          <t>9.2折</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>7.6折</t>
+          <t>8.8折</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>6.7折</t>
+          <t>7.8折</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
+      <c r="B46" s="7" t="n"/>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>qwen-max</t>
+          <t>glm-5.3-flash</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Qwen Max</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>0.37</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>8.2折</t>
+          <t>9.2折</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>7.6折</t>
+          <t>8.8折</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>6.7折</t>
+          <t>7.8折</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>阿里云·通义</t>
+        </is>
+      </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>qwen-plus</t>
+          <t>qwen-flash</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Qwen Plus</t>
+          <t>Qwen Flash</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
           <t>0.40</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -2632,27 +2632,27 @@
       <c r="B48" s="6" t="n"/>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>qwen-turbo</t>
+          <t>qwen-max</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Qwen Turbo</t>
+          <t>Qwen Max</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -2676,27 +2676,27 @@
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>qwen3.5-flash</t>
+          <t>qwen-plus</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.5 Flash</t>
+          <t>Qwen Plus</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -2720,27 +2720,27 @@
       <c r="B50" s="6" t="n"/>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>qwen3.5-plus</t>
+          <t>qwen-turbo</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.5 Plus</t>
+          <t>Qwen Turbo</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -2764,27 +2764,27 @@
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>qwen3.6-flash</t>
+          <t>qwen3.5-flash</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.6 Flash</t>
+          <t>Qwen3.5 Flash</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -2808,27 +2808,27 @@
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>qwen3.6-plus</t>
+          <t>qwen3.5-plus</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.6 Plus</t>
+          <t>Qwen3.5 Plus</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -2852,27 +2852,27 @@
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>qwen3.7-flash</t>
+          <t>qwen3.6-flash</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.7 Flash</t>
+          <t>Qwen3.6 Flash</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
           <t>0.03</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>0.13</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>0.01</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -2896,27 +2896,27 @@
       <c r="B54" s="6" t="n"/>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>qwen3.7-max</t>
+          <t>qwen3.6-plus</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.7 Max</t>
+          <t>Qwen3.6 Plus</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>7.50</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -2940,27 +2940,27 @@
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>qwen3.7-plus</t>
+          <t>qwen3.7-flash</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.7 Plus</t>
+          <t>Qwen3.7 Flash</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -2981,30 +2981,30 @@
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
-      <c r="B56" s="7" t="n"/>
+      <c r="B56" s="6" t="n"/>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>qwen3.8-max</t>
+          <t>qwen3.7-max</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max</t>
+          <t>Qwen3.7 Max</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -3025,49 +3025,45 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>GK</t>
-        </is>
-      </c>
+      <c r="B57" s="6" t="n"/>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>grok-4.5</t>
+          <t>qwen3.7-plus</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Grok 4.5</t>
+          <t>Qwen3.7 Plus</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>6.2折</t>
+          <t>8.2折</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>7.6折</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>5.5折</t>
+          <t>6.7折</t>
         </is>
       </c>
     </row>
@@ -3076,253 +3072,257 @@
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="4" t="inlineStr">
         <is>
+          <t>qwen3.8-max</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Qwen3.8 Max</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>8.2折</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>7.6折</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>6.7折</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>grok-4.5</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Grok 4.5</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>6.2折</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>6折</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>5.5折</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n"/>
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
           <t>grok-4.6</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>Grok 4.6</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>2.00</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>6.00</t>
         </is>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="G60" s="5" t="inlineStr">
         <is>
           <t>0.50</t>
         </is>
       </c>
-      <c r="H58" s="5" t="inlineStr">
+      <c r="H60" s="5" t="inlineStr">
         <is>
           <t>6.2折</t>
         </is>
       </c>
-      <c r="I58" s="5" t="inlineStr">
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>6折</t>
         </is>
       </c>
-      <c r="J58" s="5" t="inlineStr">
+      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>5.5折</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="7" t="n"/>
-      <c r="B59" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="7" t="n"/>
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>其他</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>codex-auto-review</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>Codex Auto Review</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>1.30</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F61" s="5" t="inlineStr">
         <is>
           <t>7.80</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="G61" s="5" t="inlineStr">
         <is>
           <t>0.13</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr">
+      <c r="H61" s="5" t="inlineStr">
         <is>
           <t>6.2折</t>
         </is>
       </c>
-      <c r="I59" s="5" t="inlineStr">
+      <c r="I61" s="5" t="inlineStr">
         <is>
           <t>6折</t>
         </is>
       </c>
-      <c r="J59" s="5" t="inlineStr">
+      <c r="J61" s="5" t="inlineStr">
         <is>
           <t>5.5折</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>生图</t>
         </is>
       </c>
-      <c r="B60" s="9" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>gpt-image-2</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="D62" s="9" t="inlineStr">
         <is>
           <t>GPT Image 2</t>
         </is>
       </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="E62" s="10" t="inlineStr">
         <is>
           <t>入 5.00 · 出 30.00 · 缓 1.25</t>
         </is>
       </c>
-      <c r="F60" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G60" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H60" s="10" t="inlineStr">
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="10" t="inlineStr">
         <is>
           <t>8.5折</t>
         </is>
       </c>
-      <c r="I60" s="10" t="inlineStr">
+      <c r="I62" s="10" t="inlineStr">
         <is>
           <t>8.2折</t>
         </is>
       </c>
-      <c r="J60" s="10" t="inlineStr">
+      <c r="J62" s="10" t="inlineStr">
         <is>
           <t>7.2折</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash-image</t>
-        </is>
-      </c>
-      <c r="D61" s="9" t="inlineStr">
-        <is>
-          <t>Gemini 2.5 Flash Image</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
-        <is>
-          <t>入 0.30 · 出 30.00</t>
-        </is>
-      </c>
-      <c r="F61" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G61" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" s="10" t="inlineStr">
-        <is>
-          <t>9折</t>
-        </is>
-      </c>
-      <c r="I61" s="10" t="inlineStr">
-        <is>
-          <t>8.7折</t>
-        </is>
-      </c>
-      <c r="J61" s="10" t="inlineStr">
-        <is>
-          <t>8.2折</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>gemini-3.1-flash-image</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="inlineStr">
-        <is>
-          <t>Gemini 3.1 Flash Image</t>
-        </is>
-      </c>
-      <c r="E62" s="10" t="inlineStr">
-        <is>
-          <t>入 0.50 · 出 60.00</t>
-        </is>
-      </c>
-      <c r="F62" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G62" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="10" t="inlineStr">
-        <is>
-          <t>9折</t>
-        </is>
-      </c>
-      <c r="I62" s="10" t="inlineStr">
-        <is>
-          <t>8.7折</t>
-        </is>
-      </c>
-      <c r="J62" s="10" t="inlineStr">
-        <is>
-          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n"/>
-      <c r="B63" s="7" t="n"/>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>gemini-3.1-flash-lite-image</t>
+          <t>gemini-2.5-flash-image</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Gemini 3.1 Flash Lite Image</t>
+          <t>Gemini 2.5 Flash Image</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
         <is>
-          <t>入 0.25 · 出 30.00</t>
+          <t>入 0.30 · 出 30.00</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
@@ -3353,24 +3353,20 @@
     </row>
     <row r="64">
       <c r="A64" s="6" t="n"/>
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>Vidu</t>
-        </is>
-      </c>
+      <c r="B64" s="6" t="n"/>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>viduq2-image</t>
+          <t>gemini-3.1-flash-image</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Vidu Q2 Image</t>
+          <t>Gemini 3.1 Flash Image</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>0.03（1K）</t>
+          <t>入 0.50 · 出 60.00</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
@@ -3385,224 +3381,228 @@
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>7.5折</t>
+          <t>9折</t>
         </is>
       </c>
       <c r="I64" s="10" t="inlineStr">
         <is>
-          <t>7折</t>
+          <t>8.7折</t>
         </is>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>6.4折</t>
+          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n"/>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="7" t="n"/>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>gemini-3.1-flash-lite-image</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Flash Lite Image</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
+        <is>
+          <t>入 0.25 · 出 30.00</t>
+        </is>
+      </c>
+      <c r="F65" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="10" t="inlineStr">
+        <is>
+          <t>9折</t>
+        </is>
+      </c>
+      <c r="I65" s="10" t="inlineStr">
+        <is>
+          <t>8.7折</t>
+        </is>
+      </c>
+      <c r="J65" s="10" t="inlineStr">
+        <is>
+          <t>8.2折</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>Vidu</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>viduq2-image</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>Vidu Q2 Image</t>
+        </is>
+      </c>
+      <c r="E66" s="10" t="inlineStr">
+        <is>
+          <t>0.03（1K）</t>
+        </is>
+      </c>
+      <c r="F66" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="10" t="inlineStr">
+        <is>
+          <t>7.5折</t>
+        </is>
+      </c>
+      <c r="I66" s="10" t="inlineStr">
+        <is>
+          <t>7折</t>
+        </is>
+      </c>
+      <c r="J66" s="10" t="inlineStr">
+        <is>
+          <t>6.4折</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n"/>
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>其他</t>
         </is>
       </c>
-      <c r="C65" s="9" t="inlineStr">
+      <c r="C67" s="9" t="inlineStr">
         <is>
           <t>grok-imagine-image-pro</t>
         </is>
       </c>
-      <c r="D65" s="9" t="inlineStr">
+      <c r="D67" s="9" t="inlineStr">
         <is>
           <t>Grok Imagine Image Pro</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>0.05（1K）</t>
         </is>
       </c>
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G65" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H65" s="10" t="inlineStr">
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="10" t="inlineStr">
         <is>
           <t>6.2折</t>
         </is>
       </c>
-      <c r="I65" s="10" t="inlineStr">
+      <c r="I67" s="10" t="inlineStr">
         <is>
           <t>6折</t>
         </is>
       </c>
-      <c r="J65" s="10" t="inlineStr">
+      <c r="J67" s="10" t="inlineStr">
         <is>
           <t>5.5折</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="7" t="n"/>
-      <c r="B66" s="7" t="n"/>
-      <c r="C66" s="9" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="7" t="n"/>
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>grok-imagine-image-quality</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D68" s="9" t="inlineStr">
         <is>
           <t>Grok Imagine Image Quality</t>
         </is>
       </c>
-      <c r="E66" s="10" t="inlineStr">
+      <c r="E68" s="10" t="inlineStr">
         <is>
           <t>0.05（1K）</t>
         </is>
       </c>
-      <c r="F66" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="10" t="inlineStr">
+      <c r="F68" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="10" t="inlineStr">
         <is>
           <t>6.2折</t>
         </is>
       </c>
-      <c r="I66" s="10" t="inlineStr">
+      <c r="I68" s="10" t="inlineStr">
         <is>
           <t>6折</t>
         </is>
       </c>
-      <c r="J66" s="10" t="inlineStr">
+      <c r="J68" s="10" t="inlineStr">
         <is>
           <t>5.5折</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="11" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>生视频</t>
         </is>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>Google</t>
         </is>
       </c>
-      <c r="C67" s="12" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
         <is>
           <t>gemini-omni-flash-preview</t>
         </is>
       </c>
-      <c r="D67" s="12" t="inlineStr">
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>Gemini Omni Flash Preview</t>
         </is>
       </c>
-      <c r="E67" s="13" t="inlineStr">
+      <c r="E69" s="13" t="inlineStr">
         <is>
           <t>1.50（输入）</t>
-        </is>
-      </c>
-      <c r="F67" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="13" t="inlineStr">
-        <is>
-          <t>9折</t>
-        </is>
-      </c>
-      <c r="I67" s="13" t="inlineStr">
-        <is>
-          <t>8.7折</t>
-        </is>
-      </c>
-      <c r="J67" s="13" t="inlineStr">
-        <is>
-          <t>8.2折</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="n"/>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="12" t="inlineStr">
-        <is>
-          <t>veo-3.1</t>
-        </is>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t>Veo 3.1</t>
-        </is>
-      </c>
-      <c r="E68" s="13" t="inlineStr">
-        <is>
-          <t>0.40（720p）</t>
-        </is>
-      </c>
-      <c r="F68" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G68" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H68" s="13" t="inlineStr">
-        <is>
-          <t>9折</t>
-        </is>
-      </c>
-      <c r="I68" s="13" t="inlineStr">
-        <is>
-          <t>8.7折</t>
-        </is>
-      </c>
-      <c r="J68" s="13" t="inlineStr">
-        <is>
-          <t>8.2折</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="6" t="n"/>
-      <c r="B69" s="6" t="n"/>
-      <c r="C69" s="12" t="inlineStr">
-        <is>
-          <t>veo-3.1-fast</t>
-        </is>
-      </c>
-      <c r="D69" s="12" t="inlineStr">
-        <is>
-          <t>Veo 3.1 Fast</t>
-        </is>
-      </c>
-      <c r="E69" s="13" t="inlineStr">
-        <is>
-          <t>0.10（720p）</t>
         </is>
       </c>
       <c r="F69" s="13" t="inlineStr">
@@ -3633,20 +3633,20 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n"/>
-      <c r="B70" s="7" t="n"/>
+      <c r="B70" s="6" t="n"/>
       <c r="C70" s="12" t="inlineStr">
         <is>
-          <t>veo-3.1-lite</t>
+          <t>veo-3.1</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Veo 3.1 Lite</t>
+          <t>Veo 3.1</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
         <is>
-          <t>0.05（720p）</t>
+          <t>0.40（720p）</t>
         </is>
       </c>
       <c r="F70" s="13" t="inlineStr">
@@ -3677,24 +3677,20 @@
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>
-      <c r="B71" s="11" t="inlineStr">
-        <is>
-          <t>字节·即梦</t>
-        </is>
-      </c>
+      <c r="B71" s="6" t="n"/>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>seedance-2.0-mini-overseas-hc-os</t>
+          <t>veo-3.1-fast</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Seedance 2.0 Mini Overseas HC</t>
+          <t>Veo 3.1 Fast</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>3.50（480p）</t>
+          <t>0.10（720p）</t>
         </is>
       </c>
       <c r="F71" s="13" t="inlineStr">
@@ -3709,36 +3705,36 @@
       </c>
       <c r="H71" s="13" t="inlineStr">
         <is>
-          <t>6.2折</t>
+          <t>9折</t>
         </is>
       </c>
       <c r="I71" s="13" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>8.7折</t>
         </is>
       </c>
       <c r="J71" s="13" t="inlineStr">
         <is>
-          <t>5.5折</t>
+          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n"/>
-      <c r="B72" s="6" t="n"/>
+      <c r="B72" s="7" t="n"/>
       <c r="C72" s="12" t="inlineStr">
         <is>
-          <t>seedance-2.0-fast-hc-os</t>
+          <t>veo-3.1-lite</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Seedance 2.0 Fast HC</t>
+          <t>Veo 3.1 Lite</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
         <is>
-          <t>5.60（480p）</t>
+          <t>0.05（720p）</t>
         </is>
       </c>
       <c r="F72" s="13" t="inlineStr">
@@ -3753,36 +3749,40 @@
       </c>
       <c r="H72" s="13" t="inlineStr">
         <is>
-          <t>8.4折</t>
+          <t>9折</t>
         </is>
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>8.1折</t>
+          <t>8.7折</t>
         </is>
       </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>7.1折</t>
+          <t>8.2折</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n"/>
-      <c r="B73" s="6" t="n"/>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>字节·即梦</t>
+        </is>
+      </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>seedance-2.0-os</t>
+          <t>seedance-2.0-mini-overseas-hc-os</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Seedance 2.0</t>
+          <t>Seedance 2.0 Mini Overseas HC</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
         <is>
-          <t>7.00（480p）</t>
+          <t>3.50（480p）</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
@@ -3797,36 +3797,36 @@
       </c>
       <c r="H73" s="13" t="inlineStr">
         <is>
-          <t>9.8折</t>
+          <t>6.2折</t>
         </is>
       </c>
       <c r="I73" s="13" t="inlineStr">
         <is>
-          <t>9.7折</t>
+          <t>6折</t>
         </is>
       </c>
       <c r="J73" s="13" t="inlineStr">
         <is>
-          <t>9.4折</t>
+          <t>5.5折</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n"/>
-      <c r="B74" s="7" t="n"/>
+      <c r="B74" s="6" t="n"/>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>seedance-2.0-overseas-hc-os</t>
+          <t>seedance-2.0-fast-hc-os</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Seedance 2.0 Overseas HC</t>
+          <t>Seedance 2.0 Fast HC</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
         <is>
-          <t>7.00（480p）</t>
+          <t>5.60（480p）</t>
         </is>
       </c>
       <c r="F74" s="13" t="inlineStr">
@@ -3841,40 +3841,36 @@
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>9.8折</t>
+          <t>8.4折</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>9.7折</t>
+          <t>8.1折</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>9.4折</t>
+          <t>7.1折</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n"/>
-      <c r="B75" s="12" t="inlineStr">
-        <is>
-          <t>MiniMax</t>
-        </is>
-      </c>
+      <c r="B75" s="6" t="n"/>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>minimax-h3</t>
+          <t>seedance-2.0-os</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>MiniMax H3</t>
+          <t>Seedance 2.0</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>0.08（768p）</t>
+          <t>7.00（480p）</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
@@ -3905,24 +3901,20 @@
     </row>
     <row r="76">
       <c r="A76" s="6" t="n"/>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>Vidu</t>
-        </is>
-      </c>
+      <c r="B76" s="7" t="n"/>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>viduq2</t>
+          <t>seedance-2.0-overseas-hc-os</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q2</t>
+          <t>Seedance 2.0 Overseas HC</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
         <is>
-          <t>首秒 0.05 + 续秒 0.01/秒 + 5s示例 0.09 + 10s示例 0.14</t>
+          <t>7.00（480p）</t>
         </is>
       </c>
       <c r="F76" s="13" t="inlineStr">
@@ -3937,36 +3929,40 @@
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>7.5折</t>
+          <t>9.8折</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>7折</t>
+          <t>9.7折</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>6.4折</t>
+          <t>9.4折</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n"/>
-      <c r="B77" s="6" t="n"/>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>viduq2-pro</t>
+          <t>minimax-h3</t>
         </is>
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q2 Pro</t>
+          <t>MiniMax H3</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>首秒 0.04 + 续秒 0.03/秒 + 5s示例 0.13 + 10s示例 0.25</t>
+          <t>0.08（768p）</t>
         </is>
       </c>
       <c r="F77" s="13" t="inlineStr">
@@ -3981,36 +3977,40 @@
       </c>
       <c r="H77" s="13" t="inlineStr">
         <is>
-          <t>7.5折</t>
+          <t>9.8折</t>
         </is>
       </c>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>7折</t>
+          <t>9.7折</t>
         </is>
       </c>
       <c r="J77" s="13" t="inlineStr">
         <is>
-          <t>6.4折</t>
+          <t>9.4折</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n"/>
-      <c r="B78" s="6" t="n"/>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>Vidu</t>
+        </is>
+      </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>viduq2-turbo</t>
+          <t>viduq2</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q2 Turbo</t>
+          <t>Vidu Q2</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
         <is>
-          <t>首秒 0.03 + 续秒 0.01/秒 + 5s示例 0.07 + 10s示例 0.12</t>
+          <t>首秒 0.05 + 续秒 0.01/秒 + 5s示例 0.09 + 10s示例 0.14</t>
         </is>
       </c>
       <c r="F78" s="13" t="inlineStr">
@@ -4044,17 +4044,17 @@
       <c r="B79" s="6" t="n"/>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>viduq3</t>
+          <t>viduq2-pro</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q3</t>
+          <t>Vidu Q2 Pro</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
         <is>
-          <t>0.04（540p）</t>
+          <t>首秒 0.04 + 续秒 0.03/秒 + 5s示例 0.13 + 10s示例 0.25</t>
         </is>
       </c>
       <c r="F79" s="13" t="inlineStr">
@@ -4088,17 +4088,17 @@
       <c r="B80" s="6" t="n"/>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>viduq3-mix</t>
+          <t>viduq2-turbo</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q3 Mix</t>
+          <t>Vidu Q2 Turbo</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
         <is>
-          <t>0.12（720p）</t>
+          <t>首秒 0.03 + 续秒 0.01/秒 + 5s示例 0.07 + 10s示例 0.12</t>
         </is>
       </c>
       <c r="F80" s="13" t="inlineStr">
@@ -4132,17 +4132,17 @@
       <c r="B81" s="6" t="n"/>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>viduq3-pro</t>
+          <t>viduq3</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q3 Pro</t>
+          <t>Vidu Q3</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
         <is>
-          <t>0.05（540p）</t>
+          <t>0.04（540p）</t>
         </is>
       </c>
       <c r="F81" s="13" t="inlineStr">
@@ -4176,17 +4176,17 @@
       <c r="B82" s="6" t="n"/>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>viduq3-pro-fast</t>
+          <t>viduq3-mix</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q3 Pro Fast</t>
+          <t>Vidu Q3 Mix</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
         <is>
-          <t>0.06（720p）</t>
+          <t>0.12（720p）</t>
         </is>
       </c>
       <c r="F82" s="13" t="inlineStr">
@@ -4217,20 +4217,20 @@
     </row>
     <row r="83">
       <c r="A83" s="6" t="n"/>
-      <c r="B83" s="7" t="n"/>
+      <c r="B83" s="6" t="n"/>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>viduq3-turbo</t>
+          <t>viduq3-pro</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>Vidu Q3 Turbo</t>
+          <t>Vidu Q3 Pro</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr">
         <is>
-          <t>0.04（540p）</t>
+          <t>0.05（540p）</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
@@ -4261,24 +4261,20 @@
     </row>
     <row r="84">
       <c r="A84" s="6" t="n"/>
-      <c r="B84" s="12" t="inlineStr">
-        <is>
-          <t>阿里云·通义</t>
-        </is>
-      </c>
+      <c r="B84" s="6" t="n"/>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>wan2.7</t>
+          <t>viduq3-pro-fast</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Wan 2.7</t>
+          <t>Vidu Q3 Pro Fast</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
         <is>
-          <t>0.10（720p）</t>
+          <t>0.06（720p）</t>
         </is>
       </c>
       <c r="F84" s="13" t="inlineStr">
@@ -4293,40 +4289,36 @@
       </c>
       <c r="H84" s="13" t="inlineStr">
         <is>
-          <t>9.2折</t>
+          <t>7.5折</t>
         </is>
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>8.8折</t>
+          <t>7折</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
         <is>
-          <t>7.8折</t>
+          <t>6.4折</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n"/>
-      <c r="B85" s="11" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
+      <c r="B85" s="7" t="n"/>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>grok-imagine-video-1.5</t>
+          <t>viduq3-turbo</t>
         </is>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>Grok Imagine Video 1.5</t>
+          <t>Vidu Q3 Turbo</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>0.08（480p）</t>
+          <t>0.04（540p）</t>
         </is>
       </c>
       <c r="F85" s="13" t="inlineStr">
@@ -4341,36 +4333,40 @@
       </c>
       <c r="H85" s="13" t="inlineStr">
         <is>
-          <t>6.2折</t>
+          <t>7.5折</t>
         </is>
       </c>
       <c r="I85" s="13" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>7折</t>
         </is>
       </c>
       <c r="J85" s="13" t="inlineStr">
         <is>
-          <t>5.5折</t>
+          <t>6.4折</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="n"/>
-      <c r="B86" s="6" t="n"/>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>阿里云·通义</t>
+        </is>
+      </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>happyhorse-1.1</t>
+          <t>wan2.7</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>HappyHorse 1.1</t>
+          <t>Wan 2.7</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
         <is>
-          <t>0.07（480p）</t>
+          <t>0.10（720p）</t>
         </is>
       </c>
       <c r="F86" s="13" t="inlineStr">
@@ -4385,103 +4381,195 @@
       </c>
       <c r="H86" s="13" t="inlineStr">
         <is>
-          <t>6.2折</t>
+          <t>9.2折</t>
         </is>
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>8.8折</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>5.5折</t>
+          <t>7.8折</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n"/>
-      <c r="B87" s="6" t="n"/>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
+          <t>grok-imagine-video-1.5</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>Grok Imagine Video 1.5</t>
+        </is>
+      </c>
+      <c r="E87" s="13" t="inlineStr">
+        <is>
+          <t>0.08（480p）</t>
+        </is>
+      </c>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H87" s="13" t="inlineStr">
+        <is>
+          <t>6.2折</t>
+        </is>
+      </c>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>6折</t>
+        </is>
+      </c>
+      <c r="J87" s="13" t="inlineStr">
+        <is>
+          <t>5.5折</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>happyhorse-1.1</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
+          <t>HappyHorse 1.1</t>
+        </is>
+      </c>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>0.07（480p）</t>
+        </is>
+      </c>
+      <c r="F88" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H88" s="13" t="inlineStr">
+        <is>
+          <t>6.2折</t>
+        </is>
+      </c>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>6折</t>
+        </is>
+      </c>
+      <c r="J88" s="13" t="inlineStr">
+        <is>
+          <t>5.5折</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
           <t>happyhorse-1.0</t>
         </is>
       </c>
-      <c r="D87" s="12" t="inlineStr">
+      <c r="D89" s="12" t="inlineStr">
         <is>
           <t>HappyHorse 1.0</t>
         </is>
       </c>
-      <c r="E87" s="13" t="inlineStr">
+      <c r="E89" s="13" t="inlineStr">
         <is>
           <t>0.07（480p）</t>
         </is>
       </c>
-      <c r="F87" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G87" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H87" s="13" t="inlineStr">
+      <c r="F89" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G89" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H89" s="13" t="inlineStr">
         <is>
           <t>8.2折</t>
         </is>
       </c>
-      <c r="I87" s="13" t="inlineStr">
+      <c r="I89" s="13" t="inlineStr">
         <is>
           <t>7.6折</t>
         </is>
       </c>
-      <c r="J87" s="13" t="inlineStr">
+      <c r="J89" s="13" t="inlineStr">
         <is>
           <t>6.7折</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="7" t="n"/>
-      <c r="B88" s="7" t="n"/>
-      <c r="C88" s="12" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="7" t="n"/>
+      <c r="B90" s="7" t="n"/>
+      <c r="C90" s="12" t="inlineStr">
         <is>
           <t>happyhorse-1.0-video-edit</t>
         </is>
       </c>
-      <c r="D88" s="12" t="inlineStr">
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>HappyHorse 1.0 Video Edit</t>
         </is>
       </c>
-      <c r="E88" s="13" t="inlineStr">
+      <c r="E90" s="13" t="inlineStr">
         <is>
           <t>0.14（720p）</t>
         </is>
       </c>
-      <c r="F88" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G88" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H88" s="13" t="inlineStr">
+      <c r="F90" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" s="13" t="inlineStr">
         <is>
           <t>8.2折</t>
         </is>
       </c>
-      <c r="I88" s="13" t="inlineStr">
+      <c r="I90" s="13" t="inlineStr">
         <is>
           <t>7.6折</t>
         </is>
       </c>
-      <c r="J88" s="13" t="inlineStr">
+      <c r="J90" s="13" t="inlineStr">
         <is>
           <t>6.7折</t>
         </is>
@@ -4489,25 +4577,25 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="B76:B83"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="B23:B33"/>
-    <mergeCell ref="B45:B56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A3:A59"/>
-    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B73:B76"/>
+    <mergeCell ref="B47:B58"/>
+    <mergeCell ref="A3:A61"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="A62:A68"/>
     <mergeCell ref="B16:B22"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="A67:A88"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="A60:A66"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="B87:B90"/>
+    <mergeCell ref="B23:B34"/>
+    <mergeCell ref="B78:B85"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="A69:A90"/>
     <mergeCell ref="B3:B15"/>
-    <mergeCell ref="B85:B88"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="B35:B38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>